<commit_message>
chore(tools): enriquece a fixture de preservacao sem depender do arquivo real
- formatado.xlsx NAO tinha formatacao condicional, validacao, autofiltro, coluna
  oculta nem formula: o primeiro criterio de aceite de H-24 passaria vazio,
  assertando a preservacao de elementos que nunca estiveram la
- --enriquecer roda sobre a fixture versionada e por isso nao exige o arquivo
  real, que build_fixtures.py normalmente consome
- idempotente, e respeita a ordem que o esquema OOXML impoe aos filhos de
  <worksheet> — fora de ordem o Excel pede reparo
</commit_message>
<xml_diff>
--- a/tests/fixtures/formatado.xlsx
+++ b/tests/fixtures/formatado.xlsx
@@ -3131,7 +3131,8 @@
     <col min="13" max="13" width="19.7109375" style="162" customWidth="1"/>
     <col min="14" max="14" width="17.5703125" style="162" customWidth="1"/>
     <col min="15" max="15" width="11.7109375" style="162" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="162"/>
+    <col min="16" max="16" width="9.140625" style="162" hidden="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="162"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -3548,8 +3549,9 @@
       <c r="M9" s="156" t="s">
         <v>26</v>
       </c>
-      <c r="N9" s="214" t="s">
-        <v>27</v>
+      <c r="N9" s="214">
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="O9" s="163">
         <v>46212</v>
@@ -3603,6 +3605,17 @@
       <c r="P10" s="279"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:P10"/>
+  <conditionalFormatting sqref="L2:L10">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="DESEMBARA">
+      <formula>NOT(ISERROR(SEARCH("DESEMBARA",L2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H10">
+      <formula1>"RIO,SC,MULTI,MULTIRIO,RO"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>

</xml_diff>